<commit_message>
feat: support updated prisma workbook columns
</commit_message>
<xml_diff>
--- a/docs/Zellot_PRISMA-Checkliste.xlsx
+++ b/docs/Zellot_PRISMA-Checkliste.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\klieb\OneDrive\Documents\01_petra\01_WIPAED\Masterarbeit\Prisma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6543266-E800-4C84-B999-CA47E5409C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE72AA0D-D940-4C64-A8C3-B754500D3982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="13763" xr2:uid="{FEA2155B-E447-4FE8-99FC-D4B00EBF6187}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{FEA2155B-E447-4FE8-99FC-D4B00EBF6187}"/>
   </bookViews>
   <sheets>
     <sheet name="PRISMA-Recherche" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="136">
   <si>
     <t>PRISMA Checkliste</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>ENTSCHEIDUNG</t>
-  </si>
-  <si>
-    <t>BEGRÜNDUNG für Einschluss oder Ausschluss</t>
   </si>
   <si>
     <t>erfüllt</t>
@@ -428,6 +425,35 @@
   </si>
   <si>
     <t>ausgeschlossen</t>
+  </si>
+  <si>
+    <t>Endbegründung für Einschluss oder Ausschluss</t>
+  </si>
+  <si>
+    <t>Begründung Phase 2 für
+Einschluss oder Ausschluss</t>
+  </si>
+  <si>
+    <t>Begründung Phase 3 für
+Einschluss oder Ausschluss</t>
+  </si>
+  <si>
+    <t>manuell überprüfen</t>
+  </si>
+  <si>
+    <t>https://www.gruene-liste-praevention.de/nano.cms/datenbank/suchen, https://abc.znl-ulm.de/, https://www.uniklinik-ulm.de/aktuelles/detailansicht/abc-achtsam-bedacht-clever.html</t>
+  </si>
+  <si>
+    <t>https://www.gruene-liste-praevention.de/nano.cms/datenbank/suchen, https://www.balu-und-du.de/, https://www.praeventionstag.de/dokumentation/download.cms?id=6601, https://www.schulministerium.nrw/balu-und-du-junge-erwachsene-engagieren-sich-fuer-grundschulkinder</t>
+  </si>
+  <si>
+    <t>https://www.gruene-liste-praevention.de/nano.cms/datenbank/suchen, https://www.xn--gewaltprvention-an-schulen-nhc.ch/index.html, https://www.gruene-liste-praevention.de/communities-that-care/Media/Steckbrief_Umsetzungsqualitat_PFADE.pdf, https://www.pgfwirkt.ch/de/projektliste/denk-wege/</t>
+  </si>
+  <si>
+    <t>https://www.gruene-liste-praevention.de/nano.cms/datenbank/suchen, https://www.ctc-info.de/communities-that-care/medien/2025/2265151000-qualitaetsstandards-denkzeit-klassisch-25.pdf, https://www.denkzeit.info/, https://www.ipip-berlin.de/fort--und-weiterbildung/denkzeit-trainingsprogramme/</t>
+  </si>
+  <si>
+    <t>https://www.gruene-liste-praevention.de/nano.cms/datenbank/suchen, https://www.ctc-info.de/communities-that-care/medien/2024/3173124501-ipsy-information-und-psychosoziale-kompetenz_-anwendbarkeit-in-foerderschulen.pdf, https://www.fsv.uni-jena.de/68365/ipsy-ein-suchtpraeventives-lebenskompetenzenprogramm, https://www.tk.de/presse/schulbasierte-suchtpraevention-2043254?tkcm=ab, https://www.gruene-liste-praevention.de/communities-that-care/Media/Steckbrief_Umsetzungsqualitat_IPSY.pdf</t>
   </si>
 </sst>
 </file>
@@ -504,7 +530,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -521,13 +547,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -890,7 +926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{146F31E4-3985-4260-95A8-4C36E247892D}">
-  <dimension ref="A1:W71"/>
+  <dimension ref="A1:AA71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="37.73046875" customWidth="1"/>
@@ -899,27 +935,30 @@
     <col min="6" max="6" width="10.6640625" style="3"/>
     <col min="7" max="8" width="14.1328125" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="26.59765625" style="3" customWidth="1"/>
-    <col min="11" max="11" width="14.6640625" customWidth="1"/>
-    <col min="12" max="12" width="18.9296875" customWidth="1"/>
-    <col min="13" max="13" width="20.73046875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.265625" customWidth="1"/>
-    <col min="15" max="15" width="17.53125" style="3" customWidth="1"/>
-    <col min="16" max="16" width="15.796875" customWidth="1"/>
-    <col min="17" max="17" width="52.3984375" customWidth="1"/>
-    <col min="18" max="18" width="15.6640625" customWidth="1"/>
-    <col min="19" max="19" width="22.53125" customWidth="1"/>
-    <col min="20" max="20" width="14.86328125" customWidth="1"/>
-    <col min="21" max="21" width="20.265625" customWidth="1"/>
-    <col min="22" max="22" width="15.1328125" customWidth="1"/>
+    <col min="10" max="11" width="26.59765625" style="10" customWidth="1"/>
+    <col min="12" max="12" width="26.59765625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" customWidth="1"/>
+    <col min="14" max="14" width="18.9296875" customWidth="1"/>
+    <col min="15" max="15" width="20.73046875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.265625" customWidth="1"/>
+    <col min="17" max="17" width="17.53125" style="10" customWidth="1"/>
+    <col min="18" max="18" width="26" style="10" customWidth="1"/>
+    <col min="19" max="19" width="26" style="3" customWidth="1"/>
+    <col min="20" max="20" width="15.796875" customWidth="1"/>
+    <col min="21" max="21" width="52.3984375" customWidth="1"/>
+    <col min="22" max="22" width="15.6640625" customWidth="1"/>
+    <col min="23" max="23" width="22.53125" customWidth="1"/>
+    <col min="24" max="24" width="14.86328125" customWidth="1"/>
+    <col min="25" max="25" width="20.265625" customWidth="1"/>
+    <col min="26" max="26" width="15.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="26.65" x14ac:dyDescent="0.85">
+    <row r="1" spans="1:27" ht="26.65" x14ac:dyDescent="0.85">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="21" x14ac:dyDescent="0.65">
+    <row r="2" spans="1:27" ht="21" x14ac:dyDescent="0.65">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -927,11 +966,11 @@
         <v>7</v>
       </c>
       <c r="H2" s="1"/>
-      <c r="K2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:27" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -942,7 +981,7 @@
         <v>3</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>4</v>
@@ -956,761 +995,788 @@
       <c r="H3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" s="6" t="s">
+      <c r="I3" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="M3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="N3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="P3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="Q3" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="P3" s="4" t="s">
+      <c r="R3" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="S3" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="T3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="Q3" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
+      <c r="U3" s="7" t="s">
+        <v>127</v>
+      </c>
       <c r="V3" s="4"/>
       <c r="W3" s="4"/>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.45">
+      <c r="X3" s="5"/>
+      <c r="Y3" s="5"/>
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4"/>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>21</v>
+      <c r="B4" s="8" t="s">
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>131</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E4" t="s">
-        <v>63</v>
+        <v>62</v>
+      </c>
+      <c r="F4" s="3">
+        <v>2026</v>
       </c>
       <c r="G4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="H4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="P4" t="str">
-        <f>IF(AND(K4="erfüllt", L4="erfüllt", M4="erfüllt", N4="erfüllt", O4="erfüllt"), "Einschluss", "Ausschluss")</f>
+      <c r="T4" t="str">
+        <f>IF(AND(M4="erfüllt", N4="erfüllt", O4="erfüllt", P4="erfüllt", Q4="erfüllt"), "Einschluss", "Ausschluss")</f>
         <v>Ausschluss</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>23</v>
+      <c r="B5" s="8" t="s">
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>62</v>
+        <v>132</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E5" t="s">
-        <v>63</v>
-      </c>
-      <c r="K5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L5" t="s">
-        <v>15</v>
+        <v>62</v>
+      </c>
+      <c r="F5" s="3">
+        <v>2011</v>
       </c>
       <c r="M5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N5" t="s">
-        <v>15</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="P5" t="str">
-        <f t="shared" ref="P5:P7" si="0">IF(AND(K5="erfüllt", L5="erfüllt", M5="erfüllt", N5="erfüllt", O5="erfüllt"), "Einschluss", "Ausschluss")</f>
+        <v>14</v>
+      </c>
+      <c r="O5" t="s">
+        <v>14</v>
+      </c>
+      <c r="P5" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="T5" t="str">
+        <f>IF(AND(M5="erfüllt", N5="erfüllt", O5="erfüllt", P5="erfüllt", Q5="erfüllt"), "Einschluss", "Ausschluss")</f>
         <v>Einschluss</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>24</v>
+      <c r="B6" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>62</v>
+        <v>133</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>63</v>
-      </c>
-      <c r="P6" t="str">
-        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+      <c r="F6" s="3">
+        <v>2011</v>
+      </c>
+      <c r="T6" t="str">
+        <f>IF(AND(M6="erfüllt", N6="erfüllt", O6="erfüllt", P6="erfüllt", Q6="erfüllt"), "Einschluss", "Ausschluss")</f>
         <v>Ausschluss</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>25</v>
+      <c r="B7" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>134</v>
       </c>
       <c r="D7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
-      </c>
-      <c r="P7" t="str">
-        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+      <c r="F7" s="3">
+        <v>2014</v>
+      </c>
+      <c r="T7" t="str">
+        <f>IF(AND(M7="erfüllt", N7="erfüllt", O7="erfüllt", P7="erfüllt", Q7="erfüllt"), "Einschluss", "Ausschluss")</f>
         <v>Ausschluss</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>5</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>26</v>
+      <c r="B8" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>135</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+      <c r="F8" s="3">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>6</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>27</v>
+      <c r="B9" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>7</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>28</v>
+      <c r="B10" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>8</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>29</v>
+      <c r="B11" s="8" t="s">
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>9</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>30</v>
+      <c r="B12" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>10</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>31</v>
+      <c r="B13" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E13" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>11</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>32</v>
+      <c r="B14" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>12</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>33</v>
+      <c r="B15" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E15" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>13</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>34</v>
+      <c r="B16" s="8" t="s">
+        <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>14</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>35</v>
+      <c r="B17" s="8" t="s">
+        <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>15</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>36</v>
+      <c r="B18" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>16</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>37</v>
+      <c r="B19" s="8" t="s">
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>17</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>38</v>
+      <c r="B20" s="8" t="s">
+        <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>18</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>39</v>
+      <c r="B21" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>19</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>40</v>
+      <c r="B22" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>20</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>41</v>
+      <c r="B23" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>21</v>
       </c>
-      <c r="B24" s="9" t="s">
-        <v>42</v>
+      <c r="B24" s="8" t="s">
+        <v>41</v>
       </c>
       <c r="C24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D24" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>22</v>
       </c>
-      <c r="B25" s="9" t="s">
-        <v>43</v>
+      <c r="B25" s="8" t="s">
+        <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>23</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>44</v>
+      <c r="B26" s="8" t="s">
+        <v>43</v>
       </c>
       <c r="C26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>24</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>45</v>
+      <c r="B27" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="C27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E27" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>25</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>46</v>
+      <c r="B28" s="8" t="s">
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D28" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>26</v>
       </c>
-      <c r="B29" s="9" t="s">
-        <v>47</v>
+      <c r="B29" s="8" t="s">
+        <v>46</v>
       </c>
       <c r="C29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>27</v>
       </c>
-      <c r="B30" s="9" t="s">
-        <v>48</v>
+      <c r="B30" s="8" t="s">
+        <v>47</v>
       </c>
       <c r="C30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>28</v>
       </c>
-      <c r="B31" s="9" t="s">
-        <v>49</v>
+      <c r="B31" s="8" t="s">
+        <v>48</v>
       </c>
       <c r="C31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E31" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>29</v>
       </c>
-      <c r="B32" s="9" t="s">
-        <v>50</v>
+      <c r="B32" s="8" t="s">
+        <v>49</v>
       </c>
       <c r="C32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D32" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E32" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>30</v>
       </c>
-      <c r="B33" s="9" t="s">
-        <v>51</v>
+      <c r="B33" s="8" t="s">
+        <v>50</v>
       </c>
       <c r="C33" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D33" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>31</v>
       </c>
-      <c r="B34" s="9" t="s">
-        <v>52</v>
+      <c r="B34" s="8" t="s">
+        <v>51</v>
       </c>
       <c r="C34" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D34" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>32</v>
       </c>
-      <c r="B35" s="9" t="s">
-        <v>53</v>
+      <c r="B35" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="C35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D35" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E35" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>33</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>54</v>
+      <c r="B36" s="8" t="s">
+        <v>53</v>
       </c>
       <c r="C36" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E36" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37">
         <v>34</v>
       </c>
-      <c r="B37" s="9" t="s">
-        <v>55</v>
+      <c r="B37" s="8" t="s">
+        <v>54</v>
       </c>
       <c r="C37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D37" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E37" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>35</v>
       </c>
-      <c r="B38" s="9" t="s">
-        <v>56</v>
+      <c r="B38" s="8" t="s">
+        <v>55</v>
       </c>
       <c r="C38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39">
         <v>36</v>
       </c>
-      <c r="B39" s="9" t="s">
-        <v>57</v>
+      <c r="B39" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="C39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E39" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40">
         <v>37</v>
       </c>
-      <c r="B40" s="9" t="s">
-        <v>58</v>
+      <c r="B40" s="8" t="s">
+        <v>57</v>
       </c>
       <c r="C40" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41">
         <v>38</v>
       </c>
-      <c r="B41" s="9" t="s">
-        <v>59</v>
+      <c r="B41" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="C41" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D41" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E41" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42">
         <v>39</v>
       </c>
-      <c r="B42" s="9" t="s">
-        <v>60</v>
+      <c r="B42" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="C42" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D42" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E42" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>40</v>
       </c>
-      <c r="B43" s="9" t="s">
-        <v>61</v>
+      <c r="B43" s="8" t="s">
+        <v>60</v>
       </c>
       <c r="C43" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D43" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.45">
@@ -1718,16 +1784,16 @@
         <v>41</v>
       </c>
       <c r="B44" t="s">
+        <v>63</v>
+      </c>
+      <c r="C44" t="s">
         <v>64</v>
       </c>
-      <c r="C44" t="s">
-        <v>65</v>
-      </c>
       <c r="D44" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E44" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.45">
@@ -1735,16 +1801,16 @@
         <v>42</v>
       </c>
       <c r="B45" t="s">
+        <v>65</v>
+      </c>
+      <c r="C45" t="s">
         <v>66</v>
       </c>
-      <c r="C45" t="s">
-        <v>67</v>
-      </c>
       <c r="D45" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E45" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.45">
@@ -1752,16 +1818,16 @@
         <v>43</v>
       </c>
       <c r="B46" t="s">
+        <v>67</v>
+      </c>
+      <c r="C46" t="s">
         <v>68</v>
       </c>
-      <c r="C46" t="s">
-        <v>69</v>
-      </c>
       <c r="D46" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.45">
@@ -1769,16 +1835,16 @@
         <v>44</v>
       </c>
       <c r="B47" t="s">
+        <v>69</v>
+      </c>
+      <c r="C47" t="s">
         <v>70</v>
       </c>
-      <c r="C47" t="s">
-        <v>71</v>
-      </c>
       <c r="D47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E47" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.45">
@@ -1786,291 +1852,291 @@
         <v>45</v>
       </c>
       <c r="B48" t="s">
+        <v>71</v>
+      </c>
+      <c r="C48" t="s">
         <v>72</v>
       </c>
-      <c r="C48" t="s">
-        <v>73</v>
-      </c>
       <c r="D48" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E48" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>46</v>
       </c>
       <c r="B49" t="s">
+        <v>73</v>
+      </c>
+      <c r="C49" t="s">
         <v>74</v>
       </c>
-      <c r="C49" t="s">
-        <v>75</v>
-      </c>
       <c r="D49" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E49" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A50">
         <v>47</v>
       </c>
       <c r="B50" t="s">
+        <v>75</v>
+      </c>
+      <c r="C50" t="s">
         <v>76</v>
       </c>
-      <c r="C50" t="s">
-        <v>77</v>
-      </c>
       <c r="D50" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E50" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A51">
         <v>48</v>
       </c>
       <c r="B51" t="s">
+        <v>77</v>
+      </c>
+      <c r="C51" t="s">
         <v>78</v>
       </c>
-      <c r="C51" t="s">
-        <v>79</v>
-      </c>
       <c r="D51" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E51" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A52">
         <v>49</v>
       </c>
       <c r="B52" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" t="s">
         <v>80</v>
       </c>
-      <c r="C52" t="s">
-        <v>81</v>
-      </c>
       <c r="D52" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E52" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>50</v>
       </c>
       <c r="B53" t="s">
+        <v>81</v>
+      </c>
+      <c r="C53" t="s">
         <v>82</v>
       </c>
-      <c r="C53" t="s">
-        <v>83</v>
-      </c>
       <c r="D53" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E53" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A54">
         <v>51</v>
       </c>
       <c r="B54" t="s">
+        <v>83</v>
+      </c>
+      <c r="C54" t="s">
         <v>84</v>
       </c>
-      <c r="C54" t="s">
-        <v>85</v>
-      </c>
       <c r="D54" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E54" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A55">
         <v>52</v>
       </c>
       <c r="B55" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C55" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D55" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E55" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A56">
         <v>53</v>
       </c>
       <c r="B56" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C56" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D56" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E56" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A57">
         <v>54</v>
       </c>
       <c r="B57" t="s">
+        <v>86</v>
+      </c>
+      <c r="C57" t="s">
         <v>87</v>
       </c>
-      <c r="C57" t="s">
-        <v>88</v>
-      </c>
       <c r="D57" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E57" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A58">
         <v>55</v>
       </c>
       <c r="B58" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C58" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D58" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E58" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>56</v>
       </c>
       <c r="B59" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C59" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D59" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E59" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A60">
         <v>57</v>
       </c>
       <c r="B60" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C60" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D60" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E60" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>58</v>
       </c>
       <c r="B61" t="s">
+        <v>96</v>
+      </c>
+      <c r="C61" t="s">
         <v>97</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
+        <v>101</v>
+      </c>
+      <c r="E61" t="s">
+        <v>62</v>
+      </c>
+      <c r="N61" t="s">
         <v>98</v>
       </c>
-      <c r="D61" t="s">
-        <v>102</v>
-      </c>
-      <c r="E61" t="s">
-        <v>63</v>
-      </c>
-      <c r="L61" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.45">
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A62">
         <v>59</v>
       </c>
       <c r="B62" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C62" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D62" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E62" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.45">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A63">
         <v>60</v>
       </c>
       <c r="B63" t="s">
+        <v>105</v>
+      </c>
+      <c r="C63" t="s">
         <v>106</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
+        <v>101</v>
+      </c>
+      <c r="E63" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A64">
+        <v>61</v>
+      </c>
+      <c r="B64" t="s">
         <v>107</v>
       </c>
-      <c r="D63" t="s">
-        <v>102</v>
-      </c>
-      <c r="E63" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A64">
-        <v>61</v>
-      </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
         <v>108</v>
       </c>
-      <c r="C64" t="s">
-        <v>109</v>
-      </c>
       <c r="D64" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.45">
@@ -2078,16 +2144,16 @@
         <v>62</v>
       </c>
       <c r="B65" t="s">
+        <v>109</v>
+      </c>
+      <c r="C65" t="s">
         <v>110</v>
       </c>
-      <c r="C65" t="s">
-        <v>111</v>
-      </c>
       <c r="D65" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E65" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.45">
@@ -2095,16 +2161,16 @@
         <v>63</v>
       </c>
       <c r="B66" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C66" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D66" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E66" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.45">
@@ -2112,16 +2178,16 @@
         <v>64</v>
       </c>
       <c r="B67" t="s">
+        <v>113</v>
+      </c>
+      <c r="C67" t="s">
         <v>114</v>
       </c>
-      <c r="C67" t="s">
-        <v>115</v>
-      </c>
       <c r="D67" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E67" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.45">
@@ -2129,16 +2195,16 @@
         <v>65</v>
       </c>
       <c r="B68" t="s">
+        <v>115</v>
+      </c>
+      <c r="C68" t="s">
         <v>116</v>
       </c>
-      <c r="C68" t="s">
-        <v>117</v>
-      </c>
       <c r="D68" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E68" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.45">
@@ -2146,16 +2212,16 @@
         <v>66</v>
       </c>
       <c r="B69" t="s">
+        <v>117</v>
+      </c>
+      <c r="C69" t="s">
         <v>118</v>
       </c>
-      <c r="C69" t="s">
-        <v>119</v>
-      </c>
       <c r="D69" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E69" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.45">
@@ -2163,16 +2229,16 @@
         <v>67</v>
       </c>
       <c r="B70" t="s">
+        <v>119</v>
+      </c>
+      <c r="C70" t="s">
         <v>120</v>
       </c>
-      <c r="C70" t="s">
-        <v>121</v>
-      </c>
       <c r="D70" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E70" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.45">
@@ -2180,43 +2246,43 @@
         <v>68</v>
       </c>
       <c r="B71" t="s">
+        <v>121</v>
+      </c>
+      <c r="C71" t="s">
         <v>122</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>123</v>
       </c>
-      <c r="D71" t="s">
-        <v>124</v>
-      </c>
       <c r="E71" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J4:J1048576">
+  <conditionalFormatting sqref="J4:L1048576">
     <cfRule type="beginsWith" dxfId="2" priority="3" operator="beginsWith" text="ein">
       <formula>LEFT(J4,LEN("ein"))="ein"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P4:P1048576">
+  <conditionalFormatting sqref="T4:T1048576">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Ein">
-      <formula>NOT(ISERROR(SEARCH("Ein",P4)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Ein",T4)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W4:W1048576">
+  <conditionalFormatting sqref="AA4:AA1048576">
     <cfRule type="beginsWith" dxfId="0" priority="2" operator="beginsWith" text="Ein">
-      <formula>LEFT(W4,LEN("Ein"))="Ein"</formula>
+      <formula>LEFT(AA4,LEN("Ein"))="Ein"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J4:J1048576" xr:uid="{93C82257-822E-45BB-AC0B-AB65FC935D30}">
       <formula1>"eingeschlossen,ausgeschlossen"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4:O1048576" xr:uid="{0FE5CD14-99AE-4CC1-A50D-B5DE0BD84DA8}">
-      <formula1>"erfüllt,nicht erfüllt"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:I1048576" xr:uid="{DC568DDD-3B6B-4A69-85C5-28EC72FEC331}">
       <formula1>"Ja,Nein"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4:Q1048576" xr:uid="{0FE5CD14-99AE-4CC1-A50D-B5DE0BD84DA8}">
+      <formula1>"erfüllt,nicht erfüllt"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>